<commit_message>
normalizing tables bonds and trading data
</commit_message>
<xml_diff>
--- a/bond_var_report.xlsx
+++ b/bond_var_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D178"/>
+  <dimension ref="A1:D171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.1808</v>
+        <v>-0.1806</v>
       </c>
       <c r="D11" t="n">
         <v>-0.2692</v>
@@ -621,3006 +621,2880 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RU000A108FX8</t>
+          <t>RU000A1089K2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ЕСЭГ1PC5</t>
+          <t>РУСАЛ 1Р7</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.1808</v>
+        <v>-0.1789</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.2692</v>
+        <v>-0.2373</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RU000A1089K2</t>
+          <t>RU000A103TL5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>РУСАЛ 1Р7</t>
+          <t>СберИОС409</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.1789</v>
+        <v>-0.1731</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.2373</v>
+        <v>-0.3491</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RU000A1089K2</t>
+          <t>RU000A10CEM1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>РУСАЛ 1Р7</t>
+          <t>ВТБС1-1600</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.1789</v>
+        <v>-0.1726</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.2373</v>
+        <v>-0.1959</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RU000A103TL5</t>
+          <t>RU000A108PZ2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>СберИОС409</t>
+          <t>Газпн3P12R</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-0.1731</v>
+        <v>-0.17</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.3491</v>
+        <v>-0.2265</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RU000A10CEM1</t>
+          <t>RU000A10DMD1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ВТБС1-1600</t>
+          <t>ВТБ Б1-386</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.1726</v>
+        <v>-0.1558</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1959</v>
+        <v>-0.1679</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RU000A108PZ2</t>
+          <t>RU000A107AS1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Газпн3P12R</t>
+          <t>ГПБ004Р01</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-0.1706</v>
+        <v>-0.1494</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.2265</v>
+        <v>-0.2251</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RU000A108PZ2</t>
+          <t>RU000A1095B8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Газпн3P12R</t>
+          <t>ИнвОбл09</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-0.1706</v>
+        <v>-0.1471</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.2265</v>
+        <v>-0.4586</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RU000A10DMD1</t>
+          <t>RU000A0NX2N4</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ВТБ Б1-386</t>
+          <t>ВТБ С1-733</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-0.1558</v>
+        <v>-0.1309</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1679</v>
+        <v>-0.3824</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RU000A107AS1</t>
+          <t>RU000A103U10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ГПБ004Р01</t>
+          <t>ВТБ Б1-246</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-0.1494</v>
+        <v>-0.1247</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.2251</v>
+        <v>-0.2197</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RU000A1095B8</t>
+          <t>RU000A10D5F8</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ИнвОбл09</t>
+          <t>СовкомБИ07</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-0.1471</v>
+        <v>-0.1237</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.4586</v>
+        <v>-0.1279</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RU000A0NX2N4</t>
+          <t>RU000A103174</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ВТБ С1-733</t>
+          <t>ВТБ Б1-217</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-0.1309</v>
+        <v>-0.1193</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.3824</v>
+        <v>-0.1394</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RU000A103U10</t>
+          <t>RU000A107407</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ВТБ Б1-246</t>
+          <t>ВТБ С1-800</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-0.1247</v>
+        <v>-0.113</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.2197</v>
+        <v>-0.3761</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RU000A10D5F8</t>
+          <t>RU000A107C75</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>СовкомБИ07</t>
+          <t>ИнвОбл01</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-0.1237</v>
+        <v>-0.1092</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1279</v>
+        <v>-0.2387</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RU000A103174</t>
+          <t>RU000A10D699</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ВТБ Б1-217</t>
+          <t>ВТБ Б1-384</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-0.1193</v>
+        <v>-0.1052</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.1394</v>
+        <v>-0.1235</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RU000A10BWL7</t>
+          <t>RU000A109775</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>МОНОП 1P05</t>
+          <t>ИнвОбл10</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>-0.1131</v>
+        <v>-0.1023</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.4995</v>
+        <v>-0.6019</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RU000A107407</t>
+          <t>RU000A0JWVT5</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ВТБ С1-800</t>
+          <t>РЕСОЛизБ05</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>-0.113</v>
+        <v>-0.09719999999999999</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.3761</v>
+        <v>-0.5658</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RU000A107C75</t>
+          <t>RU000A1040T6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ИнвОбл01</t>
+          <t>СберИОС488</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>-0.1092</v>
+        <v>-0.0958</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.2387</v>
+        <v>-0.1485</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RU000A10D699</t>
+          <t>RU000A103Y57</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ВТБ Б1-384</t>
+          <t>СберИОС485</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>-0.1052</v>
+        <v>-0.0911</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.1235</v>
+        <v>-0.3381</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RU000A109775</t>
+          <t>RU000A1043H5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ИнвОбл10</t>
+          <t>СберИОС492</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>-0.1023</v>
+        <v>-0.09089999999999999</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.6019</v>
+        <v>-0.1096</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RU000A0JWVT5</t>
+          <t>RU000A1040U4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>РЕСОЛизБ05</t>
+          <t>СберИОС489</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>-0.09719999999999999</v>
+        <v>-0.0895</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.5658</v>
+        <v>-0.1124</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RU000A1040T6</t>
+          <t>RU000A1034H4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>СберИОС488</t>
+          <t>ВТБ Б1-227</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>-0.0958</v>
+        <v>-0.0895</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.1485</v>
+        <v>-0.3636</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RU000A103Y57</t>
+          <t>RU000A0JX2F6</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>СберИОС485</t>
+          <t>ТбанкБ11</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-0.0911</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.3381</v>
+        <v>-0.1705</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RU000A1043H5</t>
+          <t>RU000A1041N7</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>СберИОС492</t>
+          <t>СберИОС491</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-0.09089999999999999</v>
+        <v>-0.08690000000000001</v>
       </c>
       <c r="D34" t="n">
-        <v>-0.1096</v>
+        <v>-0.1944</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RU000A1040U4</t>
+          <t>RU000A103166</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>СберИОС489</t>
+          <t>ВТБ Б1-216</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>-0.0895</v>
+        <v>-0.08649999999999999</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1124</v>
+        <v>-0.1299</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>RU000A1034H4</t>
+          <t>RU000A103UR0</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ВТБ Б1-227</t>
+          <t>СберИОС478</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>-0.0895</v>
+        <v>-0.0863</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.3636</v>
+        <v>-0.2188</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>RU000A0JX2F6</t>
+          <t>RU000A10D9Q7</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ТбанкБ11</t>
+          <t>СберИОС768</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.0827</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.1705</v>
+        <v>-0.0872</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>RU000A1041N7</t>
+          <t>RU000A1047M6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>СберИОС491</t>
+          <t>СберИОС502</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-0.08690000000000001</v>
+        <v>-0.0796</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.1944</v>
+        <v>-0.2337</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>RU000A103166</t>
+          <t>RU000A10CEJ7</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ВТБ Б1-216</t>
+          <t>ВТБС1-1597</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>-0.08649999999999999</v>
+        <v>-0.07829999999999999</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.1299</v>
+        <v>-0.08699999999999999</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RU000A103UR0</t>
+          <t>RU000A103P25</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>СберИОС478</t>
+          <t>СберИОС468</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-0.0863</v>
+        <v>-0.077</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.2188</v>
+        <v>-0.319</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RU000A10D9Q7</t>
+          <t>RU000A103X90</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>СберИОС768</t>
+          <t>СберИОС481</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>-0.0827</v>
+        <v>-0.0728</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.0872</v>
+        <v>-0.5237000000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>RU000A1047M6</t>
+          <t>RU000A104B04</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>СберИОС502</t>
+          <t>Петснаб1Р1</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>-0.0796</v>
+        <v>-0.06510000000000001</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.2337</v>
+        <v>-0.1533</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>RU000A10CEJ7</t>
+          <t>RU000A109YM0</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ВТБС1-1597</t>
+          <t>ГПБ004Р13</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>-0.07829999999999999</v>
+        <v>-0.0612</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.1525</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RU000A103P25</t>
+          <t>RU000A103Y16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>СберИОС468</t>
+          <t>СберИОС482</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>-0.077</v>
+        <v>-0.0593</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.319</v>
+        <v>-0.1587</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>RU000A103X90</t>
+          <t>RU000A103VP2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>СберИОС481</t>
+          <t>СберИОС479</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>-0.0728</v>
+        <v>-0.0583</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.5237000000000001</v>
+        <v>-0.08890000000000001</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>RU000A104B04</t>
+          <t>RU000A109EG4</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Петснаб1Р1</t>
+          <t>ГПБ004Р12</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>-0.06510000000000001</v>
+        <v>-0.0547</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1533</v>
+        <v>-0.1052</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RU000A109YM0</t>
+          <t>RU000A103RV8</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ГПБ004Р13</t>
+          <t>СберИОС472</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>-0.0612</v>
+        <v>-0.0521</v>
       </c>
       <c r="D47" t="n">
-        <v>-0.1525</v>
+        <v>-0.1323</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>RU000A103Y16</t>
+          <t>RU000A0JX355</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>СберИОС482</t>
+          <t>Роснфт1P2</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>-0.0593</v>
+        <v>-0.0504</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.1587</v>
+        <v>-0.1112</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>RU000A103VP2</t>
+          <t>RU000A1044Y8</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>СберИОС479</t>
+          <t>СберИОС495</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>-0.0583</v>
+        <v>-0.049</v>
       </c>
       <c r="D49" t="n">
-        <v>-0.08890000000000001</v>
+        <v>-0.1233</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RU000A109EG4</t>
+          <t>RU000A1045F4</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ГПБ004Р12</t>
+          <t>СберИОС493</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>-0.0547</v>
+        <v>-0.0483</v>
       </c>
       <c r="D50" t="n">
-        <v>-0.1052</v>
+        <v>-0.1296</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>RU000A103RV8</t>
+          <t>RU000A10D681</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>СберИОС472</t>
+          <t>ВТБ Б1-383</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>-0.0521</v>
+        <v>-0.0483</v>
       </c>
       <c r="D51" t="n">
-        <v>-0.1323</v>
+        <v>-0.0534</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RU000A0JX355</t>
+          <t>RU000A0JTW83</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Роснфт1P2</t>
+          <t>ДОМ.РФ25об</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>-0.0504</v>
+        <v>-0.0466</v>
       </c>
       <c r="D52" t="n">
-        <v>-0.1112</v>
+        <v>-0.0496</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RU000A1044Y8</t>
+          <t>RU000A1018M7</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>СберИОС495</t>
+          <t>СОПФ ФПФ 1</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>-0.049</v>
+        <v>-0.0459</v>
       </c>
       <c r="D53" t="n">
-        <v>-0.1233</v>
+        <v>-0.09379999999999999</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RU000A1045F4</t>
+          <t>RU000A103PF5</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>СберИОС493</t>
+          <t>СберИОС469</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>-0.0483</v>
+        <v>-0.0459</v>
       </c>
       <c r="D54" t="n">
-        <v>-0.1296</v>
+        <v>-0.061</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>RU000A10D681</t>
+          <t>RU000A1044W2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ВТБ Б1-383</t>
+          <t>СберИОС497</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>-0.0483</v>
+        <v>-0.0423</v>
       </c>
       <c r="D55" t="n">
-        <v>-0.0534</v>
+        <v>-0.2121</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RU000A0JTW83</t>
+          <t>RU000A0JX2D1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ДОМ.РФ25об</t>
+          <t>ТбанкБ12</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>-0.0466</v>
+        <v>-0.0389</v>
       </c>
       <c r="D56" t="n">
-        <v>-0.0496</v>
+        <v>-0.0423</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>RU000A1018M7</t>
+          <t>RU000A1044X0</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>СОПФ ФПФ 1</t>
+          <t>СберИОС496</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>-0.0459</v>
+        <v>-0.0378</v>
       </c>
       <c r="D57" t="n">
-        <v>-0.09379999999999999</v>
+        <v>-0.1892</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>RU000A103PF5</t>
+          <t>RU000A103UP4</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>СберИОС469</t>
+          <t>СберИОС476</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-0.0459</v>
+        <v>-0.0362</v>
       </c>
       <c r="D58" t="n">
-        <v>-0.061</v>
+        <v>-0.0791</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>RU000A1044W2</t>
+          <t>RU000A106XQ9</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>СберИОС497</t>
+          <t>СберИОС586</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>-0.0423</v>
+        <v>-0.0358</v>
       </c>
       <c r="D59" t="n">
-        <v>-0.2121</v>
+        <v>-0.1144</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>RU000A0JX2D1</t>
+          <t>RU000A10D327</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ТбанкБ12</t>
+          <t>ВТБ Б1-382</t>
         </is>
       </c>
       <c r="C60" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="D60" t="n">
         <v>-0.0389</v>
-      </c>
-      <c r="D60" t="n">
-        <v>-0.0423</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>RU000A1044X0</t>
+          <t>RU000A1071U9</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>СберИОС496</t>
+          <t>ЭлемЛиз1P6</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-0.0378</v>
+        <v>-0.0287</v>
       </c>
       <c r="D61" t="n">
-        <v>-0.1892</v>
+        <v>-0.1073</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>RU000A103UP4</t>
+          <t>RU000A1071Z8</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>СберИОС476</t>
+          <t>АйДиКоле05</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>-0.0362</v>
+        <v>-0.0287</v>
       </c>
       <c r="D62" t="n">
-        <v>-0.0791</v>
+        <v>-0.1704</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>RU000A106XQ9</t>
+          <t>RU000A0JX132</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>СберИОС586</t>
+          <t>Роснфт1P1</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>-0.0358</v>
+        <v>-0.0267</v>
       </c>
       <c r="D63" t="n">
-        <v>-0.1144</v>
+        <v>-0.0395</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>RU000A10D327</t>
+          <t>RU000A1047N4</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ВТБ Б1-382</t>
+          <t>СберИОС501</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>-0.035</v>
+        <v>-0.0263</v>
       </c>
       <c r="D64" t="n">
-        <v>-0.0389</v>
+        <v>-0.08790000000000001</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RU000A1071U9</t>
+          <t>RU000A107G22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ЭлемЛиз1P6</t>
+          <t>КОРПСАН 01</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>-0.0287</v>
+        <v>-0.0242</v>
       </c>
       <c r="D65" t="n">
-        <v>-0.1073</v>
+        <v>-0.4126</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>RU000A1071Z8</t>
+          <t>RU000A103UQ2</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>АйДиКоле05</t>
+          <t>СберИОС477</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>-0.0287</v>
+        <v>-0.0236</v>
       </c>
       <c r="D66" t="n">
-        <v>-0.1704</v>
+        <v>-0.0432</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>RU000A0JX132</t>
+          <t>RU000A10CX78</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Роснфт1P1</t>
+          <t>СберИОС763</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>-0.0267</v>
+        <v>-0.0236</v>
       </c>
       <c r="D67" t="n">
-        <v>-0.0395</v>
+        <v>-0.0521</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>RU000A1047N4</t>
+          <t>RU000A104A05</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>СберИОС501</t>
+          <t>Интерскол1</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>-0.0263</v>
+        <v>-0.0233</v>
       </c>
       <c r="D68" t="n">
-        <v>-0.08790000000000001</v>
+        <v>-0.1087</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RU000A107G22</t>
+          <t>RU000A1041M9</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>КОРПСАН 01</t>
+          <t>СберИОС490</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>-0.0242</v>
+        <v>-0.0229</v>
       </c>
       <c r="D69" t="n">
-        <v>-0.4126</v>
+        <v>-0.0567</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>RU000A103UQ2</t>
+          <t>RU000A103TN1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>СберИОС477</t>
+          <t>СберИОС418</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>-0.0236</v>
+        <v>-0.0204</v>
       </c>
       <c r="D70" t="n">
-        <v>-0.0432</v>
+        <v>-0.0381</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>RU000A10CX78</t>
+          <t>RU000A103RU0</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>СберИОС763</t>
+          <t>СберИОС471</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>-0.0236</v>
+        <v>-0.0202</v>
       </c>
       <c r="D71" t="n">
-        <v>-0.0521</v>
+        <v>-0.0599</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>RU000A104A05</t>
+          <t>RU000A1079H9</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Интерскол1</t>
+          <t>РоялКапБ10</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>-0.0233</v>
+        <v>-0.0201</v>
       </c>
       <c r="D72" t="n">
-        <v>-0.1087</v>
+        <v>-0.1131</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>RU000A1041M9</t>
+          <t>RU000A10AFT7</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>СберИОС490</t>
+          <t>ТелХолБ2-7</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>-0.0229</v>
+        <v>-0.0197</v>
       </c>
       <c r="D73" t="n">
-        <v>-0.0567</v>
+        <v>-0.0529</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>RU000A103TN1</t>
+          <t>RU000A104CF1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>СберИОС418</t>
+          <t>СолЛиз01</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>-0.0204</v>
+        <v>-0.0196</v>
       </c>
       <c r="D74" t="n">
-        <v>-0.0381</v>
+        <v>-0.2265</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>RU000A103RU0</t>
+          <t>RU000A0JWYJ0</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>СберИОС471</t>
+          <t>Самолет 01</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>-0.0202</v>
+        <v>-0.0195</v>
       </c>
       <c r="D75" t="n">
-        <v>-0.0599</v>
+        <v>-0.1292</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>RU000A1079H9</t>
+          <t>RU000A1075R6</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>РоялКапБ10</t>
+          <t>РегПрод1Р4</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>-0.0201</v>
+        <v>-0.0187</v>
       </c>
       <c r="D76" t="n">
-        <v>-0.1131</v>
+        <v>-0.0535</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>RU000A10AFT7</t>
+          <t>RU000A103Y40</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ТелХолБ2-7</t>
+          <t>СберИОС484</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>-0.0197</v>
+        <v>-0.0183</v>
       </c>
       <c r="D77" t="n">
-        <v>-0.0529</v>
+        <v>-0.1068</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>RU000A104CF1</t>
+          <t>RU000A107EE3</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>СолЛиз01</t>
+          <t>СОБИЛИЗ1Р4</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>-0.0196</v>
+        <v>-0.0182</v>
       </c>
       <c r="D78" t="n">
-        <v>-0.2265</v>
+        <v>-0.0941</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>RU000A0JWYJ0</t>
+          <t>RU000A107G63</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Самолет 01</t>
+          <t>ДжетЛ БО-1</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>-0.0195</v>
+        <v>-0.0177</v>
       </c>
       <c r="D79" t="n">
-        <v>-0.1292</v>
+        <v>-0.0623</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>RU000A1075R6</t>
+          <t>RU000A109TG2</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>РегПрод1Р4</t>
+          <t>iКарРус1P4</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>-0.0187</v>
+        <v>-0.0173</v>
       </c>
       <c r="D80" t="n">
-        <v>-0.0535</v>
+        <v>-0.0539</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>RU000A103Y40</t>
+          <t>RU000A1078Y6</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>СберИОС484</t>
+          <t>ЭконЛиз1Р6</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>-0.0183</v>
+        <v>-0.0164</v>
       </c>
       <c r="D81" t="n">
-        <v>-0.1068</v>
+        <v>-0.0755</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>RU000A107EE3</t>
+          <t>RU000A104DZ7</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>СОБИЛИЗ1Р4</t>
+          <t>СНХТ БО-02</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>-0.0182</v>
+        <v>-0.0163</v>
       </c>
       <c r="D82" t="n">
-        <v>-0.0941</v>
+        <v>-0.0895</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>RU000A107G63</t>
+          <t>RU000A10AHE5</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ДжетЛ БО-1</t>
+          <t>НовТех1Р2</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-0.0177</v>
+        <v>-0.0162</v>
       </c>
       <c r="D83" t="n">
-        <v>-0.0623</v>
+        <v>-0.0334</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>RU000A109TG2</t>
+          <t>RU000A1074E7</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>iКарРус1P4</t>
+          <t>РУССОЙЛ-01</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>-0.0173</v>
+        <v>-0.0159</v>
       </c>
       <c r="D84" t="n">
-        <v>-0.0539</v>
+        <v>-0.0597</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>RU000A1078Y6</t>
+          <t>RU000A105LS2</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ЭконЛиз1Р6</t>
+          <t>Реиннол1P2</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>-0.0164</v>
+        <v>-0.0157</v>
       </c>
       <c r="D85" t="n">
-        <v>-0.0755</v>
+        <v>-0.4084</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>RU000A104DZ7</t>
+          <t>RU000A107AZ6</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>СНХТ БО-02</t>
+          <t>Саммит 1P2</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>-0.0163</v>
+        <v>-0.0157</v>
       </c>
       <c r="D86" t="n">
-        <v>-0.0895</v>
+        <v>-0.1024</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RU000A10AHE5</t>
+          <t>RU000A104XJ9</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>НовТех1Р2</t>
+          <t>МГКЛ 1P1</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>-0.0162</v>
+        <v>-0.0157</v>
       </c>
       <c r="D87" t="n">
-        <v>-0.0334</v>
+        <v>-0.0764</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>RU000A1074E7</t>
+          <t>RU000A10ACF3</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>РУССОЙЛ-01</t>
+          <t>ВЭБ2Р-48</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>-0.0159</v>
+        <v>-0.0156</v>
       </c>
       <c r="D88" t="n">
-        <v>-0.0597</v>
+        <v>-0.0926</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>RU000A105LS2</t>
+          <t>RU000A107BH2</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Реиннол1P2</t>
+          <t>ИЛСБО-1-1Р</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>-0.0157</v>
+        <v>-0.0156</v>
       </c>
       <c r="D89" t="n">
-        <v>-0.4084</v>
+        <v>-0.0375</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>RU000A107AZ6</t>
+          <t>RU000A107F07</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Саммит 1P2</t>
+          <t>Унител БО1</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>-0.0157</v>
+        <v>-0.0154</v>
       </c>
       <c r="D90" t="n">
-        <v>-0.1024</v>
+        <v>-0.0897</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>RU000A104XJ9</t>
+          <t>RU000A100WF7</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>МГКЛ 1P1</t>
+          <t>Новосиб10</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>-0.0157</v>
+        <v>-0.0153</v>
       </c>
       <c r="D91" t="n">
-        <v>-0.0764</v>
+        <v>-0.6339</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RU000A10ACF3</t>
+          <t>RU000A103WB0</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ВЭБ2Р-48</t>
+          <t>СлавЭКО1Р1</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>-0.0156</v>
+        <v>-0.0149</v>
       </c>
       <c r="D92" t="n">
-        <v>-0.0926</v>
+        <v>-0.0914</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>RU000A107BH2</t>
+          <t>RU000A107EW5</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ИЛСБО-1-1Р</t>
+          <t>Джой 1P1</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>-0.0156</v>
+        <v>-0.0149</v>
       </c>
       <c r="D93" t="n">
-        <v>-0.0375</v>
+        <v>-0.077</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>RU000A107F07</t>
+          <t>RU000A10AA10</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Унител БО1</t>
+          <t>ПСБЛизП01</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>-0.0154</v>
+        <v>-0.0146</v>
       </c>
       <c r="D94" t="n">
-        <v>-0.0897</v>
+        <v>-0.028</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>RU000A100WF7</t>
+          <t>RU000A1078H1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Новосиб10</t>
+          <t>СОБИЛИЗ1Р3</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>-0.0153</v>
+        <v>-0.0146</v>
       </c>
       <c r="D95" t="n">
-        <v>-0.6339</v>
+        <v>-0.0994</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>RU000A103WB0</t>
+          <t>RU000A1079G1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>СлавЭКО1Р1</t>
+          <t>МаниКап1Р2</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>-0.0149</v>
+        <v>-0.0146</v>
       </c>
       <c r="D96" t="n">
-        <v>-0.0914</v>
+        <v>-0.0421</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>RU000A107EW5</t>
+          <t>RU000A101NG2</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Джой 1P1</t>
+          <t>МТС 1P-15</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-0.0149</v>
+        <v>-0.0143</v>
       </c>
       <c r="D97" t="n">
-        <v>-0.077</v>
+        <v>-0.0896</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>RU000A10AA10</t>
+          <t>RU000A107720</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ПСБЛизП01</t>
+          <t>МКЛизинг1</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-0.0146</v>
+        <v>-0.0142</v>
       </c>
       <c r="D98" t="n">
-        <v>-0.028</v>
+        <v>-0.102</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>RU000A1078H1</t>
+          <t>RU000A107C91</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>СОБИЛИЗ1Р3</t>
+          <t>МСБЛиз3P02</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>-0.0146</v>
+        <v>-0.014</v>
       </c>
       <c r="D99" t="n">
-        <v>-0.0994</v>
+        <v>-0.0968</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>RU000A1079G1</t>
+          <t>RU000A108TU5</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>МаниКап1Р2</t>
+          <t>Джи-гр 2Р4</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-0.0146</v>
+        <v>-0.0137</v>
       </c>
       <c r="D100" t="n">
-        <v>-0.0421</v>
+        <v>-0.0296</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>RU000A101NG2</t>
+          <t>RU000A1070A3</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>МТС 1P-15</t>
+          <t>ОхтаГрБП03</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-0.0143</v>
+        <v>-0.0136</v>
       </c>
       <c r="D101" t="n">
-        <v>-0.0896</v>
+        <v>-0.0634</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>RU000A107720</t>
+          <t>RU000A104EP6</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>МКЛизинг1</t>
+          <t>НЗРМ БО-01</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-0.0142</v>
+        <v>-0.0135</v>
       </c>
       <c r="D102" t="n">
-        <v>-0.102</v>
+        <v>-0.1502</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>RU000A107C91</t>
+          <t>RU000A109U97</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>МСБЛиз3P02</t>
+          <t>ДОМ 2P5</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-0.014</v>
+        <v>-0.0134</v>
       </c>
       <c r="D103" t="n">
-        <v>-0.0968</v>
+        <v>-0.0405</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>RU000A108TU5</t>
+          <t>RU000A1016N9</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Джи-гр 2Р4</t>
+          <t>СвердлОбл6</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>-0.0137</v>
+        <v>-0.0134</v>
       </c>
       <c r="D104" t="n">
-        <v>-0.0296</v>
+        <v>-0.7322</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>RU000A1070A3</t>
+          <t>RU000A10DFJ2</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ОхтаГрБП03</t>
+          <t>РСХБ2Р31</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-0.0136</v>
+        <v>-0.0134</v>
       </c>
       <c r="D105" t="n">
-        <v>-0.0634</v>
+        <v>-0.0233</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>RU000A104EP6</t>
+          <t>RU000A107C34</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>НЗРМ БО-01</t>
+          <t>АйДиКоле06</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>-0.0135</v>
+        <v>-0.0134</v>
       </c>
       <c r="D106" t="n">
-        <v>-0.1502</v>
+        <v>-0.0983</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>RU000A109U97</t>
+          <t>RU000A10AHB1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ДОМ 2P5</t>
+          <t>НовТех1Р1</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-0.0134</v>
+        <v>-0.0132</v>
       </c>
       <c r="D107" t="n">
-        <v>-0.0405</v>
+        <v>-0.0283</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>RU000A1016N9</t>
+          <t>RU000A1010B7</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>СвердлОбл6</t>
+          <t>ТрнфБО1P13</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-0.0134</v>
+        <v>-0.0132</v>
       </c>
       <c r="D108" t="n">
-        <v>-0.7322</v>
+        <v>-0.0374</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>RU000A10DFJ2</t>
+          <t>RU000A0ZZQH9</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>РСХБ2Р31</t>
+          <t>СвердлОбл5</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-0.0134</v>
+        <v>-0.0131</v>
       </c>
       <c r="D109" t="n">
-        <v>-0.0233</v>
+        <v>-0.7221</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>RU000A107C34</t>
+          <t>RU000A107GJ7</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>АйДиКоле06</t>
+          <t>ВсИнстр1Р1</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-0.0134</v>
+        <v>-0.013</v>
       </c>
       <c r="D110" t="n">
-        <v>-0.0983</v>
+        <v>-0.0521</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>RU000A10AHB1</t>
+          <t>RU000A106B51</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>НовТех1Р1</t>
+          <t>БДеньг-2P2</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>-0.0132</v>
+        <v>-0.0129</v>
       </c>
       <c r="D111" t="n">
-        <v>-0.0283</v>
+        <v>-0.0305</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>RU000A1010B7</t>
+          <t>RU000A109S91</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ТрнфБО1P13</t>
+          <t>РСетиМР1P7</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-0.0132</v>
+        <v>-0.0128</v>
       </c>
       <c r="D112" t="n">
-        <v>-0.0374</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>RU000A0ZZQH9</t>
+          <t>RU000A107A28</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>СвердлОбл5</t>
+          <t>sГПБ005P1P</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-0.0131</v>
+        <v>-0.0126</v>
       </c>
       <c r="D113" t="n">
-        <v>-0.7221</v>
+        <v>-0.06950000000000001</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>RU000A107GJ7</t>
+          <t>RU000A104A39</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>ВсИнстр1Р1</t>
+          <t>sКапиталР1</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-0.013</v>
+        <v>-0.0126</v>
       </c>
       <c r="D114" t="n">
-        <v>-0.0521</v>
+        <v>-0.0693</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>RU000A106B51</t>
+          <t>RU000A1074N8</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>БДеньг-2P2</t>
+          <t>ПрактЛК1Р2</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-0.0129</v>
+        <v>-0.0125</v>
       </c>
       <c r="D115" t="n">
-        <v>-0.0305</v>
+        <v>-0.1015</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>RU000A109S91</t>
+          <t>RU000A0JWYQ5</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>РСетиМР1P7</t>
+          <t>СистемБ1P4</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-0.0128</v>
+        <v>-0.0123</v>
       </c>
       <c r="D116" t="n">
-        <v>-0.03</v>
+        <v>-0.1349</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>RU000A107A28</t>
+          <t>RU000A10AHP1</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>sГПБ005P1P</t>
+          <t>ВТБФ БО-01</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-0.0126</v>
+        <v>-0.0122</v>
       </c>
       <c r="D117" t="n">
-        <v>-0.06950000000000001</v>
+        <v>-0.0354</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>RU000A104A39</t>
+          <t>RU000A1074F4</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>sКапиталР1</t>
+          <t>МаниКап1Р1</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-0.0126</v>
+        <v>-0.012</v>
       </c>
       <c r="D118" t="n">
-        <v>-0.0693</v>
+        <v>-0.0335</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>RU000A1074N8</t>
+          <t>RU000A10AHJ4</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>ПрактЛК1Р2</t>
+          <t>iПозитивР2</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-0.0125</v>
+        <v>-0.0119</v>
       </c>
       <c r="D119" t="n">
-        <v>-0.1015</v>
+        <v>-0.0235</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>RU000A0JWYQ5</t>
+          <t>RU000A10C8K3</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>СистемБ1P4</t>
+          <t>ВОКСИС-04</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-0.0123</v>
+        <v>-0.0119</v>
       </c>
       <c r="D120" t="n">
-        <v>-0.1349</v>
+        <v>-0.0368</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>RU000A10AHP1</t>
+          <t>RU000A107EP9</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>ВТБФ БО-01</t>
+          <t>СмартФ1Р02</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-0.0122</v>
+        <v>-0.0118</v>
       </c>
       <c r="D121" t="n">
-        <v>-0.0354</v>
+        <v>-0.0921</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RU000A1074F4</t>
+          <t>RU000A107795</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>МаниКап1Р1</t>
+          <t>ЛаймЗайм04</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-0.012</v>
+        <v>-0.0113</v>
       </c>
       <c r="D122" t="n">
-        <v>-0.0335</v>
+        <v>-0.1616</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RU000A10AHJ4</t>
+          <t>RU000A107225</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>iПозитивР2</t>
+          <t>АФАНСБО-01</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-0.0119</v>
+        <v>-0.0112</v>
       </c>
       <c r="D123" t="n">
-        <v>-0.0235</v>
+        <v>-0.0462</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>RU000A10C8K3</t>
+          <t>RU000A1010D3</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ВОКСИС-04</t>
+          <t>Якут-13 об</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-0.0119</v>
+        <v>-0.0108</v>
       </c>
       <c r="D124" t="n">
-        <v>-0.0368</v>
+        <v>-0.3064</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RU000A107EP9</t>
+          <t>RU000A1077X0</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>СмартФ1Р02</t>
+          <t>ИнтЛиз1Р07</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-0.0118</v>
+        <v>-0.0105</v>
       </c>
       <c r="D125" t="n">
-        <v>-0.0921</v>
+        <v>-0.0993</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>RU000A107795</t>
+          <t>RU000A104362</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ЛаймЗайм04</t>
+          <t>ВСК 1P-02R</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-0.0113</v>
+        <v>-0.0104</v>
       </c>
       <c r="D126" t="n">
-        <v>-0.1616</v>
+        <v>-0.0718</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>RU000A107225</t>
+          <t>RU000A0ZYKJ1</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>АФАНСБО-01</t>
+          <t>СПбГО35002</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>-0.0112</v>
+        <v>-0.0103</v>
       </c>
       <c r="D127" t="n">
-        <v>-0.0462</v>
+        <v>-0.7409</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>RU000A1010D3</t>
+          <t>RU000A1011B5</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Якут-13 об</t>
+          <t>КраснодКр3</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-0.0108</v>
+        <v>-0.0102</v>
       </c>
       <c r="D128" t="n">
-        <v>-0.3064</v>
+        <v>-0.5775</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>RU000A1077X0</t>
+          <t>RU000A105MP6</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ИнтЛиз1Р07</t>
+          <t>ДФФ 2Р-01</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-0.0105</v>
+        <v>-0.0098</v>
       </c>
       <c r="D129" t="n">
-        <v>-0.0993</v>
+        <v>-0.11</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>RU000A104362</t>
+          <t>RU000A10A7H3</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>ВСК 1P-02R</t>
+          <t>СибурХ1Р02</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-0.0104</v>
+        <v>-0.0098</v>
       </c>
       <c r="D130" t="n">
-        <v>-0.0718</v>
+        <v>-0.021</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>RU000A0ZYKJ1</t>
+          <t>RU000A107AW3</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>СПбГО35002</t>
+          <t>Аэрфью2Р02</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-0.0103</v>
+        <v>-0.0095</v>
       </c>
       <c r="D131" t="n">
-        <v>-0.7409</v>
+        <v>-0.0475</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>RU000A1011B5</t>
+          <t>RU000A1040S8</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>КраснодКр3</t>
+          <t>Ульоб34004</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-0.0102</v>
+        <v>-0.009299999999999999</v>
       </c>
       <c r="D132" t="n">
-        <v>-0.5775</v>
+        <v>-0.4315</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>RU000A105MP6</t>
+          <t>RU000A10A6J1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>ДФФ 2Р-01</t>
+          <t>ТомскАдм 9</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-0.0098</v>
+        <v>-0.009299999999999999</v>
       </c>
       <c r="D133" t="n">
-        <v>-0.11</v>
+        <v>-0.0284</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>RU000A10A7H3</t>
+          <t>RU000A107AM4</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>СибурХ1Р02</t>
+          <t>АЛЬФАБ2Р25</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-0.0098</v>
+        <v>-0.0089</v>
       </c>
       <c r="D134" t="n">
-        <v>-0.021</v>
+        <v>-0.0414</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RU000A107AW3</t>
+          <t>RU000A107GV2</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Аэрфью2Р02</t>
+          <t>СКЛиз1Р01</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-0.0095</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="D135" t="n">
-        <v>-0.0475</v>
+        <v>-0.2604</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>RU000A1040S8</t>
+          <t>RU000A10A398</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Ульоб34004</t>
+          <t>СИМПЛ1Р01</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-0.009299999999999999</v>
+        <v>-0.0086</v>
       </c>
       <c r="D136" t="n">
-        <v>-0.4315</v>
+        <v>-0.0235</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>RU000A10A6J1</t>
+          <t>RU000A109ZQ8</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>ТомскАдм 9</t>
+          <t>Россет1Р14</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>-0.009299999999999999</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="D137" t="n">
-        <v>-0.0284</v>
+        <v>-0.0247</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>RU000A107AM4</t>
+          <t>RU000A1013P1</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>АЛЬФАБ2Р25</t>
+          <t>ВЭБ1P-18</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-0.0089</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D138" t="n">
-        <v>-0.0414</v>
+        <v>-0.044</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>RU000A107GV2</t>
+          <t>RU000A10AAU6</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>СКЛиз1Р01</t>
+          <t>Амур 24001</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-0.008800000000000001</v>
+        <v>-0.0083</v>
       </c>
       <c r="D139" t="n">
-        <v>-0.2604</v>
+        <v>-0.0255</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>RU000A10A398</t>
+          <t>RU000A102CR0</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>СИМПЛ1Р01</t>
+          <t>МосОб35015</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-0.0086</v>
+        <v>-0.0081</v>
       </c>
       <c r="D140" t="n">
-        <v>-0.0235</v>
+        <v>-0.8638</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>RU000A109ZQ8</t>
+          <t>RU000A1075S4</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Россет1Р14</t>
+          <t>ИКС5Фин3P2</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-0.008500000000000001</v>
+        <v>-0.008</v>
       </c>
       <c r="D141" t="n">
-        <v>-0.0247</v>
+        <v>-0.0204</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>RU000A1013P1</t>
+          <t>RU000A107C67</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>ВЭБ1P-18</t>
+          <t>НорНикЗ26Д</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.008</v>
       </c>
       <c r="D142" t="n">
-        <v>-0.044</v>
+        <v>-0.9088000000000001</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>RU000A10AAU6</t>
+          <t>RU000A0JWZY6</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Амур 24001</t>
+          <t>СистемБ1P5</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-0.0083</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="D143" t="n">
-        <v>-0.0255</v>
+        <v>-0.0407</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>RU000A102CR0</t>
+          <t>RU000A10AG22</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>МосОб35015</t>
+          <t>ЕСЭГ1PC6</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-0.0081</v>
+        <v>-0.0074</v>
       </c>
       <c r="D144" t="n">
-        <v>-0.8638</v>
+        <v>-0.0214</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>RU000A1075S4</t>
+          <t>RU000A10ADJ3</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>ИКС5Фин3P2</t>
+          <t>ЭТС 1Р06</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-0.008</v>
+        <v>-0.0073</v>
       </c>
       <c r="D145" t="n">
-        <v>-0.0204</v>
+        <v>-0.0238</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>RU000A107C67</t>
+          <t>RU000A107KR2</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>НорНикЗ26Д</t>
+          <t>МигКр 04</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-0.008</v>
+        <v>-0.0071</v>
       </c>
       <c r="D146" t="n">
-        <v>-0.9088000000000001</v>
+        <v>-0.0982</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>RU000A0JWZY6</t>
+          <t>RU000A109VM6</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>СистемБ1P5</t>
+          <t>КАМАЗ БП13</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.0067</v>
       </c>
       <c r="D147" t="n">
-        <v>-0.0407</v>
+        <v>-0.0239</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>RU000A10AG22</t>
+          <t>RU000A107456</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>ЕСЭГ1PC6</t>
+          <t>МТС-Банк03</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-0.0074</v>
+        <v>-0.0066</v>
       </c>
       <c r="D148" t="n">
-        <v>-0.0214</v>
+        <v>-0.0619</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>RU000A10ADJ3</t>
+          <t>RU000A10AFW1</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>ЭТС 1Р06</t>
+          <t>РСетиМР1P8</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-0.0073</v>
+        <v>-0.0066</v>
       </c>
       <c r="D149" t="n">
-        <v>-0.0238</v>
+        <v>-0.0221</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>RU000A107KR2</t>
+          <t>RU000A108G05</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>МигКр 04</t>
+          <t>ЕврХол3P01</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-0.0071</v>
+        <v>-0.0065</v>
       </c>
       <c r="D150" t="n">
-        <v>-0.0982</v>
+        <v>-0.0221</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>RU000A109VM6</t>
+          <t>RU000A107DP1</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>КАМАЗ БП13</t>
+          <t>РСетиМР1Р5</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-0.0067</v>
+        <v>-0.0059</v>
       </c>
       <c r="D151" t="n">
-        <v>-0.0239</v>
+        <v>-0.0186</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>RU000A107456</t>
+          <t>RU000A1070L0</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>МТС-Банк03</t>
+          <t>ЯТЭК 1P-3</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>-0.0066</v>
+        <v>-0.0058</v>
       </c>
       <c r="D152" t="n">
-        <v>-0.0619</v>
+        <v>-0.0772</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>RU000A10AFW1</t>
+          <t>RU000A105DS9</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>РСетиМР1P8</t>
+          <t>АПРИ 2Р1</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-0.0066</v>
+        <v>-0.0057</v>
       </c>
       <c r="D153" t="n">
-        <v>-0.0221</v>
+        <v>-0.0789</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>RU000A108G05</t>
+          <t>RU000A107E81</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>ЕврХол3P01</t>
+          <t>БинФарм1P3</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>-0.0065</v>
+        <v>-0.0054</v>
       </c>
       <c r="D154" t="n">
-        <v>-0.0221</v>
+        <v>-0.06859999999999999</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>RU000A107DP1</t>
+          <t>RU000A107HG1</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>РСетиМР1Р5</t>
+          <t>Газпнф3P8R</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>-0.0059</v>
+        <v>-0.0053</v>
       </c>
       <c r="D155" t="n">
-        <v>-0.0186</v>
+        <v>-0.0212</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>RU000A1070L0</t>
+          <t>RU000A107HR8</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>ЯТЭК 1P-3</t>
+          <t>АФБАНК1Р11</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>-0.0058</v>
+        <v>-0.0052</v>
       </c>
       <c r="D156" t="n">
-        <v>-0.0772</v>
+        <v>-0.0589</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>RU000A105DS9</t>
+          <t>RU000A10CXH1</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>АПРИ 2Р1</t>
+          <t>СбКИБ1P334</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-0.0057</v>
+        <v>-0.005</v>
       </c>
       <c r="D157" t="n">
-        <v>-0.0789</v>
+        <v>-0.005</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>RU000A107E81</t>
+          <t>RU000A108QA3</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>БинФарм1P3</t>
+          <t>Мегафон2P4</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-0.0054</v>
+        <v>-0.0048</v>
       </c>
       <c r="D158" t="n">
-        <v>-0.06859999999999999</v>
+        <v>-0.07140000000000001</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>RU000A107HG1</t>
+          <t>RU000A10AEB8</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Газпнф3P8R</t>
+          <t>РусГид2Р05</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-0.0053</v>
+        <v>-0.0047</v>
       </c>
       <c r="D159" t="n">
-        <v>-0.0212</v>
+        <v>-0.0215</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>RU000A107HR8</t>
+          <t>RU000A1059N9</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>АФБАНК1Р11</t>
+          <t>ЛУКОЙЛ 26</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-0.0052</v>
+        <v>-0.0046</v>
       </c>
       <c r="D160" t="n">
-        <v>-0.0589</v>
+        <v>-1.2584</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>RU000A10CXH1</t>
+          <t>RU000A107DS5</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>СбКИБ1P334</t>
+          <t>МБЭС 2P-02</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>-0.005</v>
+        <v>-0.0045</v>
       </c>
       <c r="D161" t="n">
-        <v>-0.005</v>
+        <v>-0.1121</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>RU000A108QA3</t>
+          <t>RU000A10DEM9</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Мегафон2P4</t>
+          <t>СтройДор01</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>-0.0048</v>
+        <v>-0.0045</v>
       </c>
       <c r="D162" t="n">
-        <v>-0.07140000000000001</v>
+        <v>-0.0154</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RU000A10AEB8</t>
+          <t>RU000A1071Q7</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>РусГид2Р05</t>
+          <t>MTRCSPR001</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>-0.0047</v>
+        <v>-0.0044</v>
       </c>
       <c r="D163" t="n">
-        <v>-0.0215</v>
+        <v>-0.0712</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RU000A1059N9</t>
+          <t>RU000A107B35</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>ЛУКОЙЛ 26</t>
+          <t>ВТБ Б1-346</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>-0.0046</v>
+        <v>-0.0041</v>
       </c>
       <c r="D164" t="n">
-        <v>-1.2584</v>
+        <v>-0.0207</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>RU000A107DS5</t>
+          <t>RU000A10A349</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>МБЭС 2P-02</t>
+          <t>РусГид2Р01</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>-0.0045</v>
+        <v>-0.0037</v>
       </c>
       <c r="D165" t="n">
-        <v>-0.1121</v>
+        <v>-0.0198</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>RU000A10DEM9</t>
+          <t>RU000A10DME9</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>СтройДор01</t>
+          <t>ВТБ Б1-387</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>-0.0045</v>
+        <v>-0.0031</v>
       </c>
       <c r="D166" t="n">
-        <v>-0.0154</v>
+        <v>-0.0038</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>RU000A1071Q7</t>
+          <t>RU000A10CX86</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>MTRCSPR001</t>
+          <t>СбКИБ1P325</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>-0.0044</v>
+        <v>0</v>
       </c>
       <c r="D167" t="n">
-        <v>-0.0712</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>RU000A107B35</t>
+          <t>RU000A10AEA0</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>ВТБ Б1-346</t>
+          <t>СберИОС668</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>-0.0041</v>
+        <v>0</v>
       </c>
       <c r="D168" t="n">
-        <v>-0.0207</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>SU26226RMFS9</t>
+          <t>RU000A103T70</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>ОФЗ 26226</t>
+          <t>СибурХБО08</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>-0.0038</v>
+        <v>0.0028</v>
       </c>
       <c r="D169" t="n">
-        <v>-0.0485</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SU26226RMFS9</t>
+          <t>RU000A10DMF6</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>ОФЗ 26226</t>
+          <t>ВТБ Б1-388</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>-0.0038</v>
+        <v>0.008</v>
       </c>
       <c r="D170" t="n">
-        <v>-0.0485</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>RU000A10A349</t>
+          <t>RU000A106U33</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>РусГид2Р01</t>
+          <t>ВТБ Б1-338</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>-0.0037</v>
+        <v>0.0142</v>
       </c>
       <c r="D171" t="n">
-        <v>-0.0198</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>RU000A10DME9</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>ВТБ Б1-387</t>
-        </is>
-      </c>
-      <c r="C172" t="n">
-        <v>-0.0031</v>
-      </c>
-      <c r="D172" t="n">
-        <v>-0.0038</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>SU29016RMFS1</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>ОФЗ 29016</t>
-        </is>
-      </c>
-      <c r="C173" t="n">
-        <v>-0.0007</v>
-      </c>
-      <c r="D173" t="n">
-        <v>-0.0505</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>RU000A10AEA0</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>СберИОС668</t>
-        </is>
-      </c>
-      <c r="C174" t="n">
-        <v>0</v>
-      </c>
-      <c r="D174" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>RU000A10CX86</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>СбКИБ1P325</t>
-        </is>
-      </c>
-      <c r="C175" t="n">
-        <v>0</v>
-      </c>
-      <c r="D175" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>RU000A103T70</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>СибурХБО08</t>
-        </is>
-      </c>
-      <c r="C176" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="D176" t="n">
-        <v>0.0028</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>RU000A10DMF6</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>ВТБ Б1-388</t>
-        </is>
-      </c>
-      <c r="C177" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="D177" t="n">
-        <v>0.008</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>RU000A106U33</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>ВТБ Б1-338</t>
-        </is>
-      </c>
-      <c r="C178" t="n">
-        <v>0.0142</v>
-      </c>
-      <c r="D178" t="n">
         <v>0.0083</v>
       </c>
     </row>

</xml_diff>